<commit_message>
publish: push ASD-STE100 (a203b9f)
</commit_message>
<xml_diff>
--- a/preview/ASD-STE100/testing-criteria-scorecard-unreleased-draft.xlsx
+++ b/preview/ASD-STE100/testing-criteria-scorecard-unreleased-draft.xlsx
@@ -1800,7 +1800,7 @@
     <row r="3" ht="42" customHeight="1" s="125">
       <c r="B3" s="128" t="inlineStr">
         <is>
-          <t>DRAFT — Version unreleased draft · branch ASD-STE100 · commit b96da05 (built 2026-10-26 11:10 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
+          <t>DRAFT — Version unreleased draft · branch ASD-STE100 · commit a203b9f (built 2026-10-26 11:17 PHT). Thresholds and policy values are PROPOSED — for DOH approval. Definitions, the Technical Baseline (TB-), Terminology &amp; Registry Sources (SRC-), FHIR Traceability (TR-), Indicator Definitions (IND-), Certification &amp; Revalidation rules and the Glossary are in the companion document "HIE System Validation — Technical Reference Guide" (the Reference Guide).</t>
         </is>
       </c>
     </row>
@@ -2251,7 +2251,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -7427,7 +7427,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -12410,7 +12410,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -14543,7 +14543,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -27312,7 +27312,7 @@
   <pageMargins left="0.35" right="0.35" top="0.6" bottom="0.7" header="0.511811023622047" footer="0.25"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;L&amp;7 Healthcare Interoperability Readiness Matrix for EMR Systems&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -28622,7 +28622,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -29214,7 +29214,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -32525,7 +32525,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -33710,7 +33710,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -35220,7 +35220,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -37407,7 +37407,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -42754,7 +42754,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
@@ -47004,7 +47004,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="1" scale="100" fitToHeight="0" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter>
-    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit b96da05 · built 2026-10-26 11:10 PHT</oddHeader>
+    <oddHeader>&amp;R&amp;7 Version unreleased draft · branch ASD-STE100 · commit a203b9f · built 2026-10-26 11:17 PHT</oddHeader>
     <oddFooter>&amp;C&amp;7 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>

</xml_diff>